<commit_message>
change of the dimension of the boxes
</commit_message>
<xml_diff>
--- a/boxes.xlsx
+++ b/boxes.xlsx
@@ -2,39 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fofr6825\Documents\MATLAB\Adaptive-Palletizing\Adaptive-Palletizing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ACD1108-3C98-4868-B68A-97BAB34C3E18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D14D26B-C84D-405A-892F-C54FA0ED5AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1D3690FE-5D9A-45E6-8524-1FA8AE5358A6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -69,19 +50,22 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -106,18 +90,14 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -130,7 +110,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -140,44 +120,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -204,32 +184,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -256,24 +218,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -285,176 +229,181 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCD706C-33BE-4A55-B76B-A3C3C65C63B9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.26953125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="11.26953125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.36328125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="10.1796875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.90625" style="1"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="7" width="8" customWidth="1"/>
+    <col min="8" max="8" width="8.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -497,7 +446,7 @@
         <v>0.2</v>
       </c>
       <c r="E2" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F2" s="2">
         <v>-0.65</v>
@@ -523,7 +472,7 @@
         <v>0.2</v>
       </c>
       <c r="E3" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2">
         <v>-0.65</v>
@@ -549,7 +498,7 @@
         <v>0.2</v>
       </c>
       <c r="E4" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F4" s="2">
         <v>-0.65</v>
@@ -575,7 +524,7 @@
         <v>0.2</v>
       </c>
       <c r="E5" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F5" s="2">
         <v>-0.65</v>
@@ -601,7 +550,7 @@
         <v>0.2</v>
       </c>
       <c r="E6" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F6" s="2">
         <v>-0.65</v>
@@ -627,7 +576,7 @@
         <v>0.2</v>
       </c>
       <c r="E7" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F7" s="2">
         <v>-0.65</v>
@@ -653,7 +602,7 @@
         <v>0.2</v>
       </c>
       <c r="E8" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F8" s="2">
         <v>-0.65</v>
@@ -679,7 +628,7 @@
         <v>0.2</v>
       </c>
       <c r="E9" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F9" s="2">
         <v>-0.65</v>
@@ -705,7 +654,7 @@
         <v>0.2</v>
       </c>
       <c r="E10" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F10" s="2">
         <v>-0.65</v>
@@ -731,7 +680,7 @@
         <v>0.2</v>
       </c>
       <c r="E11" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F11" s="2">
         <v>-0.65</v>
@@ -757,7 +706,7 @@
         <v>0.2</v>
       </c>
       <c r="E12" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F12" s="2">
         <v>-0.65</v>
@@ -783,7 +732,7 @@
         <v>0.2</v>
       </c>
       <c r="E13" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F13" s="2">
         <v>-0.65</v>
@@ -809,7 +758,7 @@
         <v>0.2</v>
       </c>
       <c r="E14" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F14" s="2">
         <v>-0.65</v>
@@ -835,7 +784,7 @@
         <v>0.2</v>
       </c>
       <c r="E15" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F15" s="2">
         <v>-0.65</v>
@@ -861,7 +810,7 @@
         <v>0.2</v>
       </c>
       <c r="E16" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F16" s="2">
         <v>-0.65</v>
@@ -887,7 +836,7 @@
         <v>0.2</v>
       </c>
       <c r="E17" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2">
         <v>-0.65</v>
@@ -913,7 +862,7 @@
         <v>0.2</v>
       </c>
       <c r="E18" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F18" s="2">
         <v>-0.65</v>
@@ -939,7 +888,7 @@
         <v>0.2</v>
       </c>
       <c r="E19" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F19" s="2">
         <v>-0.65</v>
@@ -965,7 +914,7 @@
         <v>0.2</v>
       </c>
       <c r="E20" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F20" s="2">
         <v>-0.65</v>
@@ -991,7 +940,7 @@
         <v>0.2</v>
       </c>
       <c r="E21" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2">
         <v>-0.65</v>
@@ -1017,7 +966,7 @@
         <v>0.2</v>
       </c>
       <c r="E22" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F22" s="2">
         <v>-0.65</v>
@@ -1043,7 +992,7 @@
         <v>0.2</v>
       </c>
       <c r="E23" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2">
         <v>-0.65</v>
@@ -1069,7 +1018,7 @@
         <v>0.2</v>
       </c>
       <c r="E24" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F24" s="2">
         <v>-0.65</v>
@@ -1095,7 +1044,7 @@
         <v>0.2</v>
       </c>
       <c r="E25" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2">
         <v>-0.65</v>
@@ -1121,7 +1070,7 @@
         <v>0.2</v>
       </c>
       <c r="E26" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F26" s="2">
         <v>-0.65</v>
@@ -1147,7 +1096,7 @@
         <v>0.2</v>
       </c>
       <c r="E27" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2">
         <v>-0.65</v>
@@ -1173,7 +1122,7 @@
         <v>0.2</v>
       </c>
       <c r="E28" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2">
         <v>-0.65</v>
@@ -1199,7 +1148,7 @@
         <v>0.2</v>
       </c>
       <c r="E29" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F29" s="2">
         <v>-0.65</v>
@@ -1225,7 +1174,7 @@
         <v>0.2</v>
       </c>
       <c r="E30" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F30" s="2">
         <v>-0.65</v>
@@ -1251,7 +1200,7 @@
         <v>0.2</v>
       </c>
       <c r="E31" s="2">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F31" s="2">
         <v>-0.65</v>
@@ -1264,7 +1213,6 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>